<commit_message>
auto: cambios de la sesion de Claude en claude/intl-post-merge
</commit_message>
<xml_diff>
--- a/private/planilla-plazo-fijo-2026.xlsx
+++ b/private/planilla-plazo-fijo-2026.xlsx
@@ -2176,7 +2176,7 @@
         <v>52</v>
       </c>
       <c r="B16" s="21">
-        <v>46302</v>
+        <v>46303</v>
       </c>
       <c r="C16" s="22">
         <v>2500000</v>
@@ -5878,7 +5878,7 @@
         <v>110</v>
       </c>
       <c r="B8" s="21">
-        <v>46302</v>
+        <v>46303</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">

</xml_diff>